<commit_message>
Update student data and lists
</commit_message>
<xml_diff>
--- a/114-2-G10自主學習發表.xlsx
+++ b/114-2-G10自主學習發表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valerie/Desktop/Canvas/117級學生升學輔導成績分析系統/自主學習報告排程與回饋/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63B194C9-C2A6-1B48-B3DB-398282A85629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EB917FD-A93B-DA4C-99BA-6793FCE4EC4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6000" yWindow="2500" windowWidth="25600" windowHeight="14900" activeTab="1" xr2:uid="{713DCAB5-AC96-2E47-8BAF-CD1E9A18DEF8}"/>
+    <workbookView xWindow="6000" yWindow="2500" windowWidth="25600" windowHeight="14900" xr2:uid="{713DCAB5-AC96-2E47-8BAF-CD1E9A18DEF8}"/>
   </bookViews>
   <sheets>
     <sheet name="1001" sheetId="1" r:id="rId1"/>
@@ -165,9 +165,6 @@
     <t>蘇雋博</t>
   </si>
   <si>
-    <t>學吉他</t>
-  </si>
-  <si>
     <t>江安妤</t>
   </si>
   <si>
@@ -490,14 +487,19 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>自學橋牌</t>
-  </si>
-  <si>
     <t>投資理財相關研究</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>學習投資理財</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>自學橋牌</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>俄文學習</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1011,7 +1013,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="17">
       <c r="A1" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
@@ -1042,7 +1044,7 @@
         <v>5</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
@@ -1103,7 +1105,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
@@ -1157,7 +1159,7 @@
         <v>11</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>12</v>
@@ -1225,10 +1227,10 @@
         <v>23</v>
       </c>
       <c r="E11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>45</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>46</v>
       </c>
       <c r="G11" s="8"/>
     </row>
@@ -1267,7 +1269,7 @@
         <v>29</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
@@ -1286,7 +1288,7 @@
         <v>31</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
@@ -1323,10 +1325,10 @@
         <v>36</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
@@ -1424,10 +1426,10 @@
         <v>40</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>41</v>
+        <v>145</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
@@ -1440,13 +1442,13 @@
         <v>26</v>
       </c>
       <c r="C22" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D22" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="E22" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
@@ -1499,13 +1501,13 @@
         <v>29</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
@@ -1518,13 +1520,13 @@
         <v>30</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>23</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F26" s="10" t="s">
         <v>22</v>
@@ -1539,13 +1541,13 @@
         <v>31</v>
       </c>
       <c r="C27" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D27" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D27" s="10" t="s">
-        <v>48</v>
-      </c>
       <c r="E27" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
@@ -1558,13 +1560,13 @@
         <v>32</v>
       </c>
       <c r="C28" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D28" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D28" s="10" t="s">
-        <v>50</v>
-      </c>
       <c r="E28" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F28" s="8"/>
       <c r="G28" s="8"/>
@@ -1577,13 +1579,13 @@
         <v>33</v>
       </c>
       <c r="C29" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D29" s="10" t="s">
-        <v>52</v>
-      </c>
       <c r="E29" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F29" s="8"/>
       <c r="G29" s="8"/>
@@ -1615,13 +1617,13 @@
         <v>35</v>
       </c>
       <c r="C31" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D31" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D31" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="E31" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F31" s="8"/>
       <c r="G31" s="8"/>
@@ -1655,13 +1657,13 @@
         <v>37</v>
       </c>
       <c r="C33" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="10" t="s">
-        <v>56</v>
-      </c>
       <c r="E33" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F33" s="8"/>
       <c r="G33" s="8"/>
@@ -1674,13 +1676,13 @@
         <v>38</v>
       </c>
       <c r="C34" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D34" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D34" s="10" t="s">
-        <v>58</v>
-      </c>
       <c r="E34" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F34" s="8"/>
       <c r="G34" s="8"/>
@@ -1693,13 +1695,13 @@
         <v>39</v>
       </c>
       <c r="C35" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="D35" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="D35" s="10" t="s">
-        <v>60</v>
-      </c>
       <c r="E35" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F35" s="8"/>
       <c r="G35" s="8"/>
@@ -1712,13 +1714,13 @@
         <v>41</v>
       </c>
       <c r="C36" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D36" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D36" s="10" t="s">
-        <v>62</v>
-      </c>
       <c r="E36" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F36" s="8"/>
       <c r="G36" s="8"/>
@@ -1731,13 +1733,13 @@
         <v>42</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F37" s="8"/>
       <c r="G37" s="8"/>
@@ -1750,13 +1752,13 @@
         <v>43</v>
       </c>
       <c r="C38" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D38" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="10" t="s">
-        <v>65</v>
-      </c>
       <c r="E38" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F38" s="8"/>
       <c r="G38" s="8"/>
@@ -1769,13 +1771,13 @@
         <v>44</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D39" s="10" t="s">
         <v>23</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F39" s="10" t="s">
         <v>22</v>
@@ -1790,13 +1792,13 @@
         <v>45</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F40" s="8"/>
       <c r="G40" s="8"/>
@@ -8523,7 +8525,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17">
       <c r="A1" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
@@ -8547,13 +8549,13 @@
         <v>1</v>
       </c>
       <c r="C2" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="11" t="s">
-        <v>68</v>
-      </c>
       <c r="E2" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F2" s="8"/>
     </row>
@@ -8565,13 +8567,13 @@
         <v>2</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="D3" s="11" t="s">
-        <v>70</v>
-      </c>
       <c r="E3" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F3" s="8"/>
     </row>
@@ -8583,13 +8585,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="D4" s="11" t="s">
-        <v>72</v>
-      </c>
       <c r="E4" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F4" s="8"/>
     </row>
@@ -8601,13 +8603,13 @@
         <v>4</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D5" s="11" t="s">
-        <v>74</v>
-      </c>
       <c r="E5" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F5" s="8"/>
     </row>
@@ -8619,13 +8621,13 @@
         <v>5</v>
       </c>
       <c r="C6" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D6" s="11" t="s">
-        <v>76</v>
-      </c>
       <c r="E6" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F6" s="8"/>
     </row>
@@ -8637,13 +8639,13 @@
         <v>6</v>
       </c>
       <c r="C7" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="D7" s="11" t="s">
-        <v>78</v>
-      </c>
       <c r="E7" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F7" s="8"/>
     </row>
@@ -8655,13 +8657,13 @@
         <v>7</v>
       </c>
       <c r="C8" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="D8" s="11" t="s">
-        <v>80</v>
-      </c>
       <c r="E8" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F8" s="8"/>
     </row>
@@ -8673,13 +8675,13 @@
         <v>8</v>
       </c>
       <c r="C9" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="11" t="s">
-        <v>82</v>
-      </c>
       <c r="E9" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F9" s="8"/>
     </row>
@@ -8691,13 +8693,13 @@
         <v>9</v>
       </c>
       <c r="C10" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="D10" s="11" t="s">
-        <v>84</v>
-      </c>
       <c r="E10" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F10" s="8"/>
     </row>
@@ -8709,13 +8711,13 @@
         <v>10</v>
       </c>
       <c r="C11" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="E11" s="10" t="s">
         <v>86</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>87</v>
       </c>
       <c r="F11" s="8"/>
     </row>
@@ -8727,13 +8729,13 @@
         <v>11</v>
       </c>
       <c r="C12" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="D12" s="11" t="s">
-        <v>89</v>
-      </c>
       <c r="E12" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F12" s="8"/>
     </row>
@@ -8745,13 +8747,13 @@
         <v>12</v>
       </c>
       <c r="C13" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D13" s="11" t="s">
-        <v>91</v>
-      </c>
       <c r="E13" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F13" s="8"/>
     </row>
@@ -8763,16 +8765,16 @@
         <v>13</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D14" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="E14" s="11" t="s">
-        <v>44</v>
-      </c>
       <c r="F14" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="17">
@@ -8783,13 +8785,13 @@
         <v>14</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D15" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="E15" s="12" t="s">
         <v>140</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>141</v>
       </c>
       <c r="F15" s="8"/>
     </row>
@@ -8801,13 +8803,13 @@
         <v>15</v>
       </c>
       <c r="C16" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="D16" s="11" t="s">
-        <v>95</v>
-      </c>
       <c r="E16" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F16" s="8"/>
     </row>
@@ -8819,13 +8821,13 @@
         <v>16</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F17" s="8"/>
     </row>
@@ -8837,13 +8839,13 @@
         <v>17</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F18" s="8"/>
     </row>
@@ -8855,13 +8857,13 @@
         <v>18</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F19" s="8"/>
     </row>
@@ -8873,13 +8875,13 @@
         <v>19</v>
       </c>
       <c r="C20" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D20" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="D20" s="11" t="s">
-        <v>99</v>
-      </c>
       <c r="E20" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F20" s="8"/>
     </row>
@@ -8891,13 +8893,13 @@
         <v>20</v>
       </c>
       <c r="C21" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="D21" s="11" t="s">
-        <v>101</v>
-      </c>
       <c r="E21" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F21" s="8"/>
     </row>
@@ -8915,10 +8917,10 @@
         <v>25</v>
       </c>
       <c r="E22" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="F22" s="11" t="s">
         <v>138</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="17">
@@ -8929,13 +8931,13 @@
         <v>22</v>
       </c>
       <c r="C23" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D23" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D23" s="11" t="s">
-        <v>103</v>
-      </c>
       <c r="E23" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F23" s="8"/>
     </row>
@@ -8947,13 +8949,13 @@
         <v>26</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F24" s="8"/>
     </row>
@@ -8965,13 +8967,13 @@
         <v>27</v>
       </c>
       <c r="C25" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="E25" s="10" t="s">
         <v>106</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>107</v>
       </c>
       <c r="F25" s="8"/>
     </row>
@@ -8983,13 +8985,13 @@
         <v>28</v>
       </c>
       <c r="C26" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D26" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="D26" s="11" t="s">
-        <v>109</v>
-      </c>
       <c r="E26" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F26" s="8"/>
     </row>
@@ -9001,13 +9003,13 @@
         <v>29</v>
       </c>
       <c r="C27" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D27" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="D27" s="11" t="s">
-        <v>111</v>
-      </c>
       <c r="E27" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F27" s="8"/>
     </row>
@@ -9019,13 +9021,13 @@
         <v>30</v>
       </c>
       <c r="C28" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D28" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="E28" s="10" t="s">
         <v>113</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>114</v>
       </c>
       <c r="F28" s="8"/>
     </row>
@@ -9037,13 +9039,13 @@
         <v>31</v>
       </c>
       <c r="C29" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="E29" s="10" t="s">
         <v>116</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>117</v>
       </c>
       <c r="F29" s="8"/>
     </row>
@@ -9055,13 +9057,13 @@
         <v>32</v>
       </c>
       <c r="C30" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="D30" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="D30" s="11" t="s">
-        <v>119</v>
-      </c>
       <c r="E30" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F30" s="8"/>
     </row>
@@ -9073,13 +9075,13 @@
         <v>33</v>
       </c>
       <c r="C31" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D31" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="D31" s="14" t="s">
-        <v>121</v>
-      </c>
       <c r="E31" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F31" s="8"/>
     </row>
@@ -9091,13 +9093,13 @@
         <v>34</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F32" s="8"/>
     </row>
@@ -9109,13 +9111,13 @@
         <v>35</v>
       </c>
       <c r="C33" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D33" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="D33" s="11" t="s">
+      <c r="E33" s="10" t="s">
         <v>123</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>124</v>
       </c>
       <c r="F33" s="8"/>
     </row>
@@ -9127,13 +9129,13 @@
         <v>36</v>
       </c>
       <c r="C34" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="D34" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="D34" s="11" t="s">
-        <v>126</v>
-      </c>
       <c r="E34" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F34" s="8"/>
     </row>
@@ -9145,13 +9147,13 @@
         <v>37</v>
       </c>
       <c r="C35" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D35" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="D35" s="11" t="s">
-        <v>128</v>
-      </c>
       <c r="E35" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F35" s="8"/>
     </row>
@@ -9163,13 +9165,13 @@
         <v>38</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F36" s="8"/>
     </row>
@@ -9181,13 +9183,13 @@
         <v>39</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F37" s="8"/>
     </row>
@@ -9199,13 +9201,13 @@
         <v>40</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F38" s="8"/>
     </row>
@@ -9217,13 +9219,13 @@
         <v>41</v>
       </c>
       <c r="C39" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="D39" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="D39" s="11" t="s">
-        <v>130</v>
-      </c>
       <c r="E39" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F39" s="8"/>
     </row>
@@ -9235,13 +9237,13 @@
         <v>42</v>
       </c>
       <c r="C40" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D40" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="D40" s="11" t="s">
-        <v>132</v>
-      </c>
       <c r="E40" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F40" s="8"/>
     </row>
@@ -9253,13 +9255,13 @@
         <v>43</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F41" s="8"/>
     </row>
@@ -9271,13 +9273,13 @@
         <v>44</v>
       </c>
       <c r="C42" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D42" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="D42" s="11" t="s">
-        <v>135</v>
-      </c>
       <c r="E42" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F42" s="8"/>
     </row>

</xml_diff>

<commit_message>
Fix topic sync overwriting CSV imports & update student grouping for MBTI topic
</commit_message>
<xml_diff>
--- a/114-2-G10自主學習發表.xlsx
+++ b/114-2-G10自主學習發表.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valerie/Desktop/Canvas/117級學生升學輔導成績分析系統/自主學習報告排程與回饋/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EB917FD-A93B-DA4C-99BA-6793FCE4EC4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCA19A8-3CB8-AC43-B8C8-CB4A88723B40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6000" yWindow="2500" windowWidth="25600" windowHeight="14900" xr2:uid="{713DCAB5-AC96-2E47-8BAF-CD1E9A18DEF8}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="14880" activeTab="1" xr2:uid="{713DCAB5-AC96-2E47-8BAF-CD1E9A18DEF8}"/>
   </bookViews>
   <sheets>
     <sheet name="1001" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="147">
   <si>
     <t>座號</t>
   </si>
@@ -366,15 +366,9 @@
     <t>林知柔</t>
   </si>
   <si>
-    <t>高中生理財與省錢小技巧</t>
-  </si>
-  <si>
     <t>邱歆宸</t>
   </si>
   <si>
-    <t>學習韓文</t>
-  </si>
-  <si>
     <t>張心妮</t>
   </si>
   <si>
@@ -406,9 +400,6 @@
   </si>
   <si>
     <t>陳意喬</t>
-  </si>
-  <si>
-    <t>紅樓夢觀後感</t>
   </si>
   <si>
     <t>蔡侑庭</t>
@@ -500,6 +491,22 @@
   </si>
   <si>
     <t>俄文學習</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>犯罪心理學</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>日文自學</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>財經金融管理</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>從MBTI熱潮看現代人的自我認同與社交心理學</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1013,7 +1020,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="17">
       <c r="A1" s="4" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
@@ -1044,7 +1051,7 @@
         <v>5</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
@@ -1105,7 +1112,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
@@ -1159,7 +1166,7 @@
         <v>11</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>12</v>
@@ -1269,7 +1276,7 @@
         <v>29</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
@@ -1288,7 +1295,7 @@
         <v>31</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
@@ -1325,10 +1332,10 @@
         <v>36</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
@@ -1426,10 +1433,10 @@
         <v>40</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
@@ -1566,7 +1573,7 @@
         <v>49</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F28" s="8"/>
       <c r="G28" s="8"/>
@@ -1585,7 +1592,7 @@
         <v>51</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F29" s="8"/>
       <c r="G29" s="8"/>
@@ -1623,7 +1630,7 @@
         <v>53</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F31" s="8"/>
       <c r="G31" s="8"/>
@@ -1663,7 +1670,7 @@
         <v>55</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F33" s="8"/>
       <c r="G33" s="8"/>
@@ -1682,7 +1689,7 @@
         <v>57</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F34" s="8"/>
       <c r="G34" s="8"/>
@@ -1701,7 +1708,7 @@
         <v>59</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F35" s="8"/>
       <c r="G35" s="8"/>
@@ -1720,7 +1727,7 @@
         <v>61</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F36" s="8"/>
       <c r="G36" s="8"/>
@@ -1758,7 +1765,7 @@
         <v>64</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F38" s="8"/>
       <c r="G38" s="8"/>
@@ -1795,10 +1802,10 @@
         <v>65</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F40" s="8"/>
       <c r="G40" s="8"/>
@@ -8525,7 +8532,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17">
       <c r="A1" s="4" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
@@ -8555,7 +8562,7 @@
         <v>67</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F2" s="8"/>
     </row>
@@ -8573,7 +8580,7 @@
         <v>69</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F3" s="8"/>
     </row>
@@ -8591,7 +8598,7 @@
         <v>71</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F4" s="8"/>
     </row>
@@ -8609,7 +8616,7 @@
         <v>73</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F5" s="8"/>
     </row>
@@ -8627,7 +8634,7 @@
         <v>75</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F6" s="8"/>
     </row>
@@ -8645,7 +8652,7 @@
         <v>77</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F7" s="8"/>
     </row>
@@ -8663,7 +8670,7 @@
         <v>79</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F8" s="8"/>
     </row>
@@ -8681,7 +8688,7 @@
         <v>81</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F9" s="8"/>
     </row>
@@ -8699,7 +8706,7 @@
         <v>83</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F10" s="8"/>
     </row>
@@ -8735,7 +8742,7 @@
         <v>88</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F12" s="8"/>
     </row>
@@ -8753,7 +8760,7 @@
         <v>90</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F13" s="8"/>
     </row>
@@ -8788,10 +8795,10 @@
         <v>92</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F15" s="8"/>
     </row>
@@ -8809,7 +8816,7 @@
         <v>94</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F16" s="8"/>
     </row>
@@ -8824,10 +8831,10 @@
         <v>95</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F17" s="8"/>
     </row>
@@ -8881,7 +8888,7 @@
         <v>98</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F20" s="8"/>
     </row>
@@ -8899,7 +8906,7 @@
         <v>100</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F21" s="8"/>
     </row>
@@ -8917,10 +8924,10 @@
         <v>25</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="17">
@@ -8937,7 +8944,7 @@
         <v>102</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F23" s="8"/>
     </row>
@@ -8952,10 +8959,10 @@
         <v>103</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F24" s="8"/>
     </row>
@@ -8987,11 +8994,11 @@
       <c r="C26" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="D26" s="11" t="s">
-        <v>108</v>
+      <c r="D26" s="13" t="s">
+        <v>143</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F26" s="8"/>
     </row>
@@ -9003,13 +9010,13 @@
         <v>29</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>110</v>
+        <v>108</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>145</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F27" s="8"/>
     </row>
@@ -9021,13 +9028,13 @@
         <v>30</v>
       </c>
       <c r="C28" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D28" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="E28" s="10" t="s">
         <v>111</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>113</v>
       </c>
       <c r="F28" s="8"/>
     </row>
@@ -9039,13 +9046,13 @@
         <v>31</v>
       </c>
       <c r="C29" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="E29" s="10" t="s">
         <v>114</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>116</v>
       </c>
       <c r="F29" s="8"/>
     </row>
@@ -9057,13 +9064,13 @@
         <v>32</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F30" s="8"/>
     </row>
@@ -9075,13 +9082,13 @@
         <v>33</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F31" s="8"/>
     </row>
@@ -9093,13 +9100,13 @@
         <v>34</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F32" s="8"/>
     </row>
@@ -9111,13 +9118,13 @@
         <v>35</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="D33" s="11" t="s">
-        <v>122</v>
+        <v>119</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>146</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="F33" s="8"/>
     </row>
@@ -9129,13 +9136,13 @@
         <v>36</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F34" s="8"/>
     </row>
@@ -9147,13 +9154,13 @@
         <v>37</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F35" s="8"/>
     </row>
@@ -9183,13 +9190,13 @@
         <v>39</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F37" s="8"/>
     </row>
@@ -9201,13 +9208,13 @@
         <v>40</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="D38" s="11" t="s">
-        <v>122</v>
+        <v>120</v>
+      </c>
+      <c r="D38" s="13" t="s">
+        <v>144</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="F38" s="8"/>
     </row>
@@ -9219,13 +9226,13 @@
         <v>41</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F39" s="8"/>
     </row>
@@ -9237,13 +9244,13 @@
         <v>42</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F40" s="8"/>
     </row>
@@ -9255,7 +9262,7 @@
         <v>43</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D41" s="11" t="s">
         <v>73</v>
@@ -9273,13 +9280,13 @@
         <v>44</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F42" s="8"/>
     </row>

</xml_diff>

<commit_message>
Fix drag and drop duplication bug, add student total count stat card, optimize UI elements and update student view UI
</commit_message>
<xml_diff>
--- a/114-2-G10自主學習發表.xlsx
+++ b/114-2-G10自主學習發表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valerie/Desktop/Canvas/117級學生升學輔導成績分析系統/自主學習報告排程與回饋/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCA19A8-3CB8-AC43-B8C8-CB4A88723B40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4250DBF8-93F4-834E-B44F-9B0513C07FA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="14880" activeTab="1" xr2:uid="{713DCAB5-AC96-2E47-8BAF-CD1E9A18DEF8}"/>
+    <workbookView xWindow="8860" yWindow="4200" windowWidth="25600" windowHeight="14880" xr2:uid="{713DCAB5-AC96-2E47-8BAF-CD1E9A18DEF8}"/>
   </bookViews>
   <sheets>
     <sheet name="1001" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="148">
   <si>
     <t>座號</t>
   </si>
@@ -507,6 +507,10 @@
   </si>
   <si>
     <t>從MBTI熱潮看現代人的自我認同與社交心理學</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>傅天語</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1092,9 +1096,6 @@
         <v>11</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="10" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1169,12 +1170,9 @@
         <v>133</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="G8" s="10" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1208,17 +1206,13 @@
         <v>12</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>10</v>
+        <v>139</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>13</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
     </row>
     <row r="11" spans="1:7" ht="17">
       <c r="A11" s="15">
@@ -1334,8 +1328,8 @@
       <c r="D16" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="E16" s="12" t="s">
-        <v>137</v>
+      <c r="E16" s="10" t="s">
+        <v>12</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
@@ -1378,9 +1372,6 @@
         <v>11</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="10" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>